<commit_message>
Edicion de responsable,observaciones y estado en archivos de cuadratura
</commit_message>
<xml_diff>
--- a/uploads/errores_importacion.xlsx
+++ b/uploads/errores_importacion.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,64 +451,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> DUPLICADO</t>
+          <t>CONFLICTO</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>39669</t>
+          <t>40228</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>934</t>
+          <t>9505</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>RPEG</t>
+          <t>RALC</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>PRUEBA</t>
+          <t>PUBLICIDAD E INVERSIONES KOBBO SPA</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Registro ya existe en la base de datos</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> DUPLICADO</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>39668</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>9523</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>RPEG</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>PRUEBA 3</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Registro ya existe en la base de datos</t>
+          <t>La OC pertenece a IMPORTADORA Y COMERCIALIZADORA PROSA CHILE SPA</t>
         </is>
       </c>
     </row>

</xml_diff>